<commit_message>
Corrige acentos dos ramais
</commit_message>
<xml_diff>
--- a/ramais.xlsx
+++ b/ramais.xlsx
@@ -621,7 +621,7 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Centro de servi?o</t>
+          <t>Centro de serviço</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -648,7 +648,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Centro de servi?o</t>
+          <t>Centro de serviço</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -675,7 +675,7 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Centro de servi?o</t>
+          <t>Centro de serviço</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Centro de servi?o</t>
+          <t>Centro de serviço</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -730,7 +730,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Centro de servi?o</t>
+          <t>Centro de serviço</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Elvis Gon?alves</t>
+          <t>Elvis Gonçalves</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1216,7 +1216,7 @@
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Expedi??o</t>
+          <t>Expedição</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Edson J?nior</t>
+          <t>Edson Júnior</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Manuten??o</t>
+          <t>Manutenção</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Mat?ria Prima</t>
+          <t>Matéria Prima</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1584,7 +1584,7 @@
     <row r="43" ht="32" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Or?amentos</t>
+          <t>Orçamentos</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
@@ -1612,7 +1612,7 @@
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Or?amentos</t>
+          <t>Orçamentos</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1639,7 +1639,7 @@
     <row r="45" ht="32" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Or?amentos</t>
+          <t>Orçamentos</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Or?amentos</t>
+          <t>Orçamentos</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Jo?o Henrique Leal</t>
+          <t>João Henrique Leal</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -1991,7 +1991,7 @@
     <row r="58" ht="32" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Produ??o</t>
+          <t>Produção</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Rog?rio Abreu</t>
+          <t>Rogério Abreu</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -2345,7 +2345,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Qualidade - Inspe??o</t>
+          <t>Qualidade - Inspeção</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -2372,7 +2372,7 @@
     <row r="72" ht="32" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Qualidade - Inspe??o</t>
+          <t>Qualidade - Inspeção</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2400,7 +2400,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Qualidade - Inspe??o</t>
+          <t>Qualidade - Inspeção</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -2538,7 +2538,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Sala Reuni?o Grande</t>
+          <t>Sala Reunião Grande</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr"/>
@@ -2557,7 +2557,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Sala Reuni?o Pequena</t>
+          <t>Sala Reunião Pequena</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
     <row r="80" ht="32" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Seguran?a do Trabalho</t>
+          <t>Segurança do Trabalho</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Supervisor de Fabrica??o</t>
+          <t>Supervisor de Fabricação</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">

</xml_diff>